<commit_message>
Marcelo: cambios propios, guardados antes de una acción de Claude (3.B.34 3.B.35)
</commit_message>
<xml_diff>
--- a/Ejercicio-3/Parte-B/3.B.35/Code/datos_3B35.xlsx
+++ b/Ejercicio-3/Parte-B/3.B.35/Code/datos_3B35.xlsx
@@ -14,6 +14,7 @@
     <sheet name="CAN_destinos_2023" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="EFTA_destinos_2023" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="NAFTA_vehiculos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="USA_importaciones" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -74181,4 +74182,569 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Importaciones de mercancías de USA por origen (millones de dólares corrientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fuente: WITS (Banco Mundial) a partir de UN Comtrade, indicador MPRT-TRD-VL (importaciones declaradas por el importador). Cálculo propio (Code/datos_comercio.py).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Año</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MEX</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CAN</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CHN</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Total (WLD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1994</v>
+      </c>
+      <c r="B5" t="n">
+        <v>50333.5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>131916.2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>41345.8</v>
+      </c>
+      <c r="E5" t="n">
+        <v>689029.9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1995</v>
+      </c>
+      <c r="B6" t="n">
+        <v>62745.6</v>
+      </c>
+      <c r="C6" t="n">
+        <v>148277.9</v>
+      </c>
+      <c r="D6" t="n">
+        <v>48505.6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>770821.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1996</v>
+      </c>
+      <c r="B7" t="n">
+        <v>74108.10000000001</v>
+      </c>
+      <c r="C7" t="n">
+        <v>159691.2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>54396.5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>817627.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1997</v>
+      </c>
+      <c r="B8" t="n">
+        <v>87119.8</v>
+      </c>
+      <c r="C8" t="n">
+        <v>171330.6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>65811.60000000001</v>
+      </c>
+      <c r="E8" t="n">
+        <v>898025.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1998</v>
+      </c>
+      <c r="B9" t="n">
+        <v>96074.60000000001</v>
+      </c>
+      <c r="C9" t="n">
+        <v>177916.4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>75094.89999999999</v>
+      </c>
+      <c r="E9" t="n">
+        <v>944350.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1999</v>
+      </c>
+      <c r="B10" t="n">
+        <v>111067.2</v>
+      </c>
+      <c r="C10" t="n">
+        <v>201433.2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>87775.10000000001</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1059220.1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B11" t="n">
+        <v>135923.1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>230816.1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>100012.9</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1217933</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2001</v>
+      </c>
+      <c r="B12" t="n">
+        <v>131334.7</v>
+      </c>
+      <c r="C12" t="n">
+        <v>216234.1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>102267.3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1140900.2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B13" t="n">
+        <v>136025.1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>212398.4</v>
+      </c>
+      <c r="D13" t="n">
+        <v>133510.4</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1200095.8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B14" t="n">
+        <v>139686.7</v>
+      </c>
+      <c r="C14" t="n">
+        <v>225035.3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>163313.9</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1302833.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B15" t="n">
+        <v>157881.9</v>
+      </c>
+      <c r="C15" t="n">
+        <v>260161.3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>210500.1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1525304.2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B16" t="n">
+        <v>172388.6</v>
+      </c>
+      <c r="C16" t="n">
+        <v>294382.3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>259836</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1734849.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B17" t="n">
+        <v>200499.7</v>
+      </c>
+      <c r="C17" t="n">
+        <v>307723.1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>305778.9</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1918997.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B18" t="n">
+        <v>212878</v>
+      </c>
+      <c r="C18" t="n">
+        <v>317481.9</v>
+      </c>
+      <c r="D18" t="n">
+        <v>340106.6</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2017120.8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B19" t="n">
+        <v>218066.2</v>
+      </c>
+      <c r="C19" t="n">
+        <v>339074.1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>356304.6</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2164834</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B20" t="n">
+        <v>178321.6</v>
+      </c>
+      <c r="C20" t="n">
+        <v>227577.4</v>
+      </c>
+      <c r="D20" t="n">
+        <v>309530.2</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1601895.8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B21" t="n">
+        <v>232251.4</v>
+      </c>
+      <c r="C21" t="n">
+        <v>280426.5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>382964.8</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1968259.9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B22" t="n">
+        <v>265113.8</v>
+      </c>
+      <c r="C22" t="n">
+        <v>317921.2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>417340.3</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2263619.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B23" t="n">
+        <v>279957.4</v>
+      </c>
+      <c r="C23" t="n">
+        <v>327502.6</v>
+      </c>
+      <c r="D23" t="n">
+        <v>444386</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2334677.7</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B24" t="n">
+        <v>283133.7</v>
+      </c>
+      <c r="C24" t="n">
+        <v>337126.1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>459107.9</v>
+      </c>
+      <c r="E24" t="n">
+        <v>2326590.2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B25" t="n">
+        <v>296855.8</v>
+      </c>
+      <c r="C25" t="n">
+        <v>354171.8</v>
+      </c>
+      <c r="D25" t="n">
+        <v>486296.2</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2410855.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B26" t="n">
+        <v>299181.8</v>
+      </c>
+      <c r="C26" t="n">
+        <v>301942.7</v>
+      </c>
+      <c r="D26" t="n">
+        <v>504028.1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>2313424.6</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B27" t="n">
+        <v>296199.9</v>
+      </c>
+      <c r="C27" t="n">
+        <v>282919.2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>481310.4</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2247167.3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B28" t="n">
+        <v>315733.5</v>
+      </c>
+      <c r="C28" t="n">
+        <v>305647.7</v>
+      </c>
+      <c r="D28" t="n">
+        <v>525764.7</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2405276.6</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B29" t="n">
+        <v>349195.2</v>
+      </c>
+      <c r="C29" t="n">
+        <v>325683.6</v>
+      </c>
+      <c r="D29" t="n">
+        <v>563203.1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2611432.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B30" t="n">
+        <v>361320.9</v>
+      </c>
+      <c r="C30" t="n">
+        <v>326628.6</v>
+      </c>
+      <c r="D30" t="n">
+        <v>472464.9</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2567492.2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B31" t="n">
+        <v>328861.8</v>
+      </c>
+      <c r="C31" t="n">
+        <v>276195.5</v>
+      </c>
+      <c r="D31" t="n">
+        <v>457164.2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2405381.6</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B32" t="n">
+        <v>388357.5</v>
+      </c>
+      <c r="C32" t="n">
+        <v>363904.7</v>
+      </c>
+      <c r="D32" t="n">
+        <v>541531.4</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2932976.1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B33" t="n">
+        <v>459177.7</v>
+      </c>
+      <c r="C33" t="n">
+        <v>446623.9</v>
+      </c>
+      <c r="D33" t="n">
+        <v>575688.1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>3372902.2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B34" t="n">
+        <v>480050.6</v>
+      </c>
+      <c r="C34" t="n">
+        <v>429604.9</v>
+      </c>
+      <c r="D34" t="n">
+        <v>448017.4</v>
+      </c>
+      <c r="E34" t="n">
+        <v>3168471.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>